<commit_message>
Embed timeline images from Excel column G image URLs.
Reserve a fixed thumbnail slot in layout so packing stays stable, and reject non-http(s) URLs with a warning.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/template_sample.xlsx
+++ b/public/template_sample.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -407,6 +407,7 @@
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -428,6 +429,9 @@
       <c r="F1" t="str">
         <v>表示スタイル</v>
       </c>
+      <c r="G1" t="str">
+        <v>画像リンク</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -439,6 +443,9 @@
       <c r="E2" t="str">
         <v>#5D4037</v>
       </c>
+      <c r="G2" t="str">
+        <v>https://placehold.co/96x72/C45C26/FFFFFF/png?text=1945</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -504,14 +511,14 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -519,6 +526,7 @@
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -540,6 +548,9 @@
       <c r="F1" t="str">
         <v>表示スタイル</v>
       </c>
+      <c r="G1" t="str">
+        <v>画像リンク</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -625,14 +636,14 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -640,6 +651,7 @@
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -661,6 +673,9 @@
       <c r="F1" t="str">
         <v>表示スタイル</v>
       </c>
+      <c r="G1" t="str">
+        <v>画像リンク</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -672,6 +687,9 @@
       <c r="E2" t="str">
         <v>#1565C0</v>
       </c>
+      <c r="G2" t="str">
+        <v>https://placehold.co/96x72/1565C0/FFFFFF/png?text=1964</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -683,6 +701,9 @@
       <c r="E3" t="str">
         <v>#2E7D32</v>
       </c>
+      <c r="G3" t="str">
+        <v>https://placehold.co/96x72/2E7D32/FFFFFF/png?text=EXPO</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -708,6 +729,9 @@
       <c r="E5" t="str">
         <v>#5B4B8A</v>
       </c>
+      <c r="G5" t="str">
+        <v>https://placehold.co/96x72/5B4B8A/FFFFFF/png?text=IT</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -725,7 +749,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>